<commit_message>
Fix copy deck: remove fixed row height so wrap text works
</commit_message>
<xml_diff>
--- a/copy-deck.xlsx
+++ b/copy-deck.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Global</t>
@@ -563,7 +563,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr"/>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Global</t>
@@ -592,7 +592,7 @@
       </c>
       <c r="G3" s="9" t="inlineStr"/>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Global</t>
@@ -621,7 +621,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr"/>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Global</t>
@@ -650,7 +650,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -679,7 +679,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -708,7 +708,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -737,7 +737,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -766,7 +766,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr"/>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -795,7 +795,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -824,7 +824,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -853,7 +853,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -882,7 +882,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr"/>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -911,7 +911,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr"/>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -940,7 +940,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr"/>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -969,7 +969,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr"/>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -998,7 +998,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr"/>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr"/>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="G19" s="9" t="inlineStr"/>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr"/>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="G21" s="9" t="inlineStr"/>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr"/>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="G23" s="9" t="inlineStr"/>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr"/>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="G25" s="9" t="inlineStr"/>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr"/>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G27" s="9" t="inlineStr"/>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr"/>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="G29" s="9" t="inlineStr"/>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr"/>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr"/>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr"/>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G33" s="9" t="inlineStr"/>
     </row>
-    <row r="34" ht="15" customHeight="1">
+    <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr"/>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G35" s="9" t="inlineStr"/>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr"/>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr"/>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr"/>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr"/>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr"/>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="G41" s="9" t="inlineStr"/>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr"/>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G43" s="9" t="inlineStr"/>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr"/>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr"/>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr"/>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="G47" s="9" t="inlineStr"/>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G48" s="5" t="inlineStr"/>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="G49" s="9" t="inlineStr"/>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr"/>
     </row>
-    <row r="51" ht="15" customHeight="1">
+    <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G51" s="9" t="inlineStr"/>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr"/>
     </row>
-    <row r="53" ht="15" customHeight="1">
+    <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="G53" s="9" t="inlineStr"/>
     </row>
-    <row r="54" ht="15" customHeight="1">
+    <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr"/>
     </row>
-    <row r="55" ht="15" customHeight="1">
+    <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr"/>
     </row>
-    <row r="56" ht="15" customHeight="1">
+    <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr"/>
     </row>
-    <row r="57" ht="15" customHeight="1">
+    <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="G57" s="9" t="inlineStr"/>
     </row>
-    <row r="58" ht="15" customHeight="1">
+    <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr"/>
     </row>
-    <row r="59" ht="15" customHeight="1">
+    <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr"/>
     </row>
-    <row r="60" ht="15" customHeight="1">
+    <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr"/>
     </row>
-    <row r="61" ht="15" customHeight="1">
+    <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr"/>
     </row>
-    <row r="62" ht="15" customHeight="1">
+    <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr"/>
     </row>
-    <row r="63" ht="15" customHeight="1">
+    <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr"/>
     </row>
-    <row r="64" ht="15" customHeight="1">
+    <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr"/>
     </row>
-    <row r="65" ht="15" customHeight="1">
+    <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr"/>
     </row>
-    <row r="66" ht="15" customHeight="1">
+    <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr"/>
     </row>
-    <row r="67" ht="15" customHeight="1">
+    <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr"/>
     </row>
-    <row r="68" ht="15" customHeight="1">
+    <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr"/>
     </row>
-    <row r="69" ht="15" customHeight="1">
+    <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr"/>
     </row>
-    <row r="70" ht="15" customHeight="1">
+    <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr"/>
     </row>
-    <row r="71" ht="15" customHeight="1">
+    <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr"/>
     </row>
-    <row r="72" ht="15" customHeight="1">
+    <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr"/>
     </row>
-    <row r="73" ht="15" customHeight="1">
+    <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr"/>
     </row>
-    <row r="74" ht="15" customHeight="1">
+    <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr"/>
     </row>
-    <row r="75" ht="15" customHeight="1">
+    <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr"/>
     </row>
-    <row r="76" ht="15" customHeight="1">
+    <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr"/>
     </row>
-    <row r="77" ht="15" customHeight="1">
+    <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr"/>
     </row>
-    <row r="78" ht="15" customHeight="1">
+    <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr"/>
     </row>
-    <row r="79" ht="15" customHeight="1">
+    <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr"/>
     </row>
-    <row r="80" ht="15" customHeight="1">
+    <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr"/>
     </row>
-    <row r="81" ht="15" customHeight="1">
+    <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr"/>
     </row>
-    <row r="82" ht="15" customHeight="1">
+    <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr"/>
     </row>
-    <row r="83" ht="15" customHeight="1">
+    <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="G83" s="9" t="inlineStr"/>
     </row>
-    <row r="84" ht="15" customHeight="1">
+    <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr"/>
     </row>
-    <row r="85" ht="15" customHeight="1">
+    <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr"/>
     </row>
-    <row r="86" ht="15" customHeight="1">
+    <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr"/>
     </row>
-    <row r="87" ht="15" customHeight="1">
+    <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr"/>
     </row>
-    <row r="88" ht="15" customHeight="1">
+    <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="G88" s="5" t="inlineStr"/>
     </row>
-    <row r="89" ht="15" customHeight="1">
+    <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr"/>
     </row>
-    <row r="90" ht="15" customHeight="1">
+    <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="G90" s="5" t="inlineStr"/>
     </row>
-    <row r="91" ht="15" customHeight="1">
+    <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr"/>
     </row>
-    <row r="92" ht="15" customHeight="1">
+    <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr"/>
     </row>
-    <row r="93" ht="15" customHeight="1">
+    <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="G93" s="9" t="inlineStr"/>
     </row>
-    <row r="94" ht="15" customHeight="1">
+    <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G94" s="5" t="inlineStr"/>
     </row>
-    <row r="95" ht="15" customHeight="1">
+    <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="G95" s="9" t="inlineStr"/>
     </row>
-    <row r="96" ht="15" customHeight="1">
+    <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G96" s="5" t="inlineStr"/>
     </row>
-    <row r="97" ht="15" customHeight="1">
+    <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="G97" s="9" t="inlineStr"/>
     </row>
-    <row r="98" ht="15" customHeight="1">
+    <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3591,7 +3591,7 @@
       </c>
       <c r="G98" s="5" t="inlineStr"/>
     </row>
-    <row r="99" ht="15" customHeight="1">
+    <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="G99" s="9" t="inlineStr"/>
     </row>
-    <row r="100" ht="15" customHeight="1">
+    <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
           <t>Work</t>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="G100" s="5" t="inlineStr"/>
     </row>
-    <row r="101" ht="15" customHeight="1">
+    <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr"/>
     </row>
-    <row r="102" ht="15" customHeight="1">
+    <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="G102" s="5" t="inlineStr"/>
     </row>
-    <row r="103" ht="15" customHeight="1">
+    <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr"/>
     </row>
-    <row r="104" ht="15" customHeight="1">
+    <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3765,7 +3765,7 @@
       </c>
       <c r="G104" s="5" t="inlineStr"/>
     </row>
-    <row r="105" ht="15" customHeight="1">
+    <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G105" s="9" t="inlineStr"/>
     </row>
-    <row r="106" ht="15" customHeight="1">
+    <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="G106" s="5" t="inlineStr"/>
     </row>
-    <row r="107" ht="15" customHeight="1">
+    <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr"/>
     </row>
-    <row r="108" ht="15" customHeight="1">
+    <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="G108" s="5" t="inlineStr"/>
     </row>
-    <row r="109" ht="15" customHeight="1">
+    <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr"/>
     </row>
-    <row r="110" ht="15" customHeight="1">
+    <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G110" s="5" t="inlineStr"/>
     </row>
-    <row r="111" ht="15" customHeight="1">
+    <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="G111" s="9" t="inlineStr"/>
     </row>
-    <row r="112" ht="15" customHeight="1">
+    <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="G112" s="5" t="inlineStr"/>
     </row>
-    <row r="113" ht="15" customHeight="1">
+    <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="G113" s="9" t="inlineStr"/>
     </row>
-    <row r="114" ht="15" customHeight="1">
+    <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="G114" s="5" t="inlineStr"/>
     </row>
-    <row r="115" ht="15" customHeight="1">
+    <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="G115" s="9" t="inlineStr"/>
     </row>
-    <row r="116" ht="15" customHeight="1">
+    <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G116" s="5" t="inlineStr"/>
     </row>
-    <row r="117" ht="15" customHeight="1">
+    <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="G117" s="9" t="inlineStr"/>
     </row>
-    <row r="118" ht="15" customHeight="1">
+    <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="G118" s="5" t="inlineStr"/>
     </row>
-    <row r="119" ht="15" customHeight="1">
+    <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="G119" s="9" t="inlineStr"/>
     </row>
-    <row r="120" ht="15" customHeight="1">
+    <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="G120" s="5" t="inlineStr"/>
     </row>
-    <row r="121" ht="15" customHeight="1">
+    <row r="121">
       <c r="A121" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="G121" s="9" t="inlineStr"/>
     </row>
-    <row r="122" ht="15" customHeight="1">
+    <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr"/>
     </row>
-    <row r="123" ht="15" customHeight="1">
+    <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr"/>
     </row>
-    <row r="124" ht="15" customHeight="1">
+    <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr"/>
     </row>
-    <row r="125" ht="15" customHeight="1">
+    <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr"/>
     </row>
-    <row r="126" ht="15" customHeight="1">
+    <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr"/>
     </row>
-    <row r="127" ht="15" customHeight="1">
+    <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="G127" s="9" t="inlineStr"/>
     </row>
-    <row r="128" ht="15" customHeight="1">
+    <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="G128" s="5" t="inlineStr"/>
     </row>
-    <row r="129" ht="15" customHeight="1">
+    <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4554,7 +4554,7 @@
       </c>
       <c r="G129" s="9" t="inlineStr"/>
     </row>
-    <row r="130" ht="15" customHeight="1">
+    <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="G130" s="5" t="inlineStr"/>
     </row>
-    <row r="131" ht="15" customHeight="1">
+    <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="G131" s="9" t="inlineStr"/>
     </row>
-    <row r="132" ht="15" customHeight="1">
+    <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4653,7 +4653,7 @@
       </c>
       <c r="G132" s="5" t="inlineStr"/>
     </row>
-    <row r="133" ht="15" customHeight="1">
+    <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="G133" s="9" t="inlineStr"/>
     </row>
-    <row r="134" ht="15" customHeight="1">
+    <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4719,7 +4719,7 @@
       </c>
       <c r="G134" s="5" t="inlineStr"/>
     </row>
-    <row r="135" ht="15" customHeight="1">
+    <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="G135" s="9" t="inlineStr"/>
     </row>
-    <row r="136" ht="15" customHeight="1">
+    <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="G136" s="5" t="inlineStr"/>
     </row>
-    <row r="137" ht="15" customHeight="1">
+    <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="G137" s="9" t="inlineStr"/>
     </row>
-    <row r="138" ht="15" customHeight="1">
+    <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="G138" s="5" t="inlineStr"/>
     </row>
-    <row r="139" ht="15" customHeight="1">
+    <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="G139" s="9" t="inlineStr"/>
     </row>
-    <row r="140" ht="15" customHeight="1">
+    <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="G140" s="5" t="inlineStr"/>
     </row>
-    <row r="141" ht="15" customHeight="1">
+    <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="G141" s="9" t="inlineStr"/>
     </row>
-    <row r="142" ht="15" customHeight="1">
+    <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="G142" s="5" t="inlineStr"/>
     </row>
-    <row r="143" ht="15" customHeight="1">
+    <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="G143" s="9" t="inlineStr"/>
     </row>
-    <row r="144" ht="15" customHeight="1">
+    <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="G144" s="5" t="inlineStr"/>
     </row>
-    <row r="145" ht="15" customHeight="1">
+    <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="G145" s="9" t="inlineStr"/>
     </row>
-    <row r="146" ht="15" customHeight="1">
+    <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G146" s="5" t="inlineStr"/>
     </row>
-    <row r="147" ht="15" customHeight="1">
+    <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="G147" s="9" t="inlineStr"/>
     </row>
-    <row r="148" ht="15" customHeight="1">
+    <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="G148" s="5" t="inlineStr"/>
     </row>
-    <row r="149" ht="15" customHeight="1">
+    <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="G149" s="9" t="inlineStr"/>
     </row>
-    <row r="150" ht="15" customHeight="1">
+    <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G150" s="5" t="inlineStr"/>
     </row>
-    <row r="151" ht="15" customHeight="1">
+    <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="G151" s="9" t="inlineStr"/>
     </row>
-    <row r="152" ht="15" customHeight="1">
+    <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="G152" s="5" t="inlineStr"/>
     </row>
-    <row r="153" ht="15" customHeight="1">
+    <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
           <t>Laura</t>
@@ -5310,7 +5310,7 @@
       </c>
       <c r="G153" s="9" t="inlineStr"/>
     </row>
-    <row r="154" ht="15" customHeight="1">
+    <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="G154" s="5" t="inlineStr"/>
     </row>
-    <row r="155" ht="15" customHeight="1">
+    <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="G155" s="9" t="inlineStr"/>
     </row>
-    <row r="156" ht="15" customHeight="1">
+    <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="G156" s="5" t="inlineStr"/>
     </row>
-    <row r="157" ht="15" customHeight="1">
+    <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="G157" s="9" t="inlineStr"/>
     </row>
-    <row r="158" ht="15" customHeight="1">
+    <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5455,7 +5455,7 @@
       </c>
       <c r="G158" s="5" t="inlineStr"/>
     </row>
-    <row r="159" ht="15" customHeight="1">
+    <row r="159">
       <c r="A159" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="G159" s="9" t="inlineStr"/>
     </row>
-    <row r="160" ht="15" customHeight="1">
+    <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5513,7 +5513,7 @@
       </c>
       <c r="G160" s="5" t="inlineStr"/>
     </row>
-    <row r="161" ht="15" customHeight="1">
+    <row r="161">
       <c r="A161" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="G161" s="9" t="inlineStr"/>
     </row>
-    <row r="162" ht="15" customHeight="1">
+    <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5575,7 +5575,7 @@
       </c>
       <c r="G162" s="5" t="inlineStr"/>
     </row>
-    <row r="163" ht="15" customHeight="1">
+    <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="G163" s="9" t="inlineStr"/>
     </row>
-    <row r="164" ht="15" customHeight="1">
+    <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="G164" s="5" t="inlineStr"/>
     </row>
-    <row r="165" ht="15" customHeight="1">
+    <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="G165" s="9" t="inlineStr"/>
     </row>
-    <row r="166" ht="15" customHeight="1">
+    <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5707,7 +5707,7 @@
       </c>
       <c r="G166" s="5" t="inlineStr"/>
     </row>
-    <row r="167" ht="15" customHeight="1">
+    <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="G167" s="9" t="inlineStr"/>
     </row>
-    <row r="168" ht="15" customHeight="1">
+    <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5773,7 +5773,7 @@
       </c>
       <c r="G168" s="5" t="inlineStr"/>
     </row>
-    <row r="169" ht="15" customHeight="1">
+    <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5806,7 +5806,7 @@
       </c>
       <c r="G169" s="9" t="inlineStr"/>
     </row>
-    <row r="170" ht="15" customHeight="1">
+    <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="G170" s="5" t="inlineStr"/>
     </row>
-    <row r="171" ht="15" customHeight="1">
+    <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="G171" s="9" t="inlineStr"/>
     </row>
-    <row r="172" ht="15" customHeight="1">
+    <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5905,7 +5905,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr"/>
     </row>
-    <row r="173" ht="15" customHeight="1">
+    <row r="173">
       <c r="A173" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -5938,7 +5938,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr"/>
     </row>
-    <row r="174" ht="15" customHeight="1">
+    <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr"/>
     </row>
-    <row r="175" ht="15" customHeight="1">
+    <row r="175">
       <c r="A175" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr"/>
     </row>
-    <row r="176" ht="15" customHeight="1">
+    <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6037,7 +6037,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr"/>
     </row>
-    <row r="177" ht="15" customHeight="1">
+    <row r="177">
       <c r="A177" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6066,7 +6066,7 @@
       </c>
       <c r="G177" s="9" t="inlineStr"/>
     </row>
-    <row r="178" ht="15" customHeight="1">
+    <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6095,7 +6095,7 @@
       </c>
       <c r="G178" s="5" t="inlineStr"/>
     </row>
-    <row r="179" ht="15" customHeight="1">
+    <row r="179">
       <c r="A179" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="G179" s="9" t="inlineStr"/>
     </row>
-    <row r="180" ht="15" customHeight="1">
+    <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6153,7 +6153,7 @@
       </c>
       <c r="G180" s="5" t="inlineStr"/>
     </row>
-    <row r="181" ht="15" customHeight="1">
+    <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="G181" s="9" t="inlineStr"/>
     </row>
-    <row r="182" ht="15" customHeight="1">
+    <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G182" s="5" t="inlineStr"/>
     </row>
-    <row r="183" ht="15" customHeight="1">
+    <row r="183">
       <c r="A183" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6244,7 +6244,7 @@
       </c>
       <c r="G183" s="9" t="inlineStr"/>
     </row>
-    <row r="184" ht="15" customHeight="1">
+    <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="G184" s="5" t="inlineStr"/>
     </row>
-    <row r="185" ht="15" customHeight="1">
+    <row r="185">
       <c r="A185" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6310,7 +6310,7 @@
       </c>
       <c r="G185" s="9" t="inlineStr"/>
     </row>
-    <row r="186" ht="15" customHeight="1">
+    <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G186" s="5" t="inlineStr"/>
     </row>
-    <row r="187" ht="15" customHeight="1">
+    <row r="187">
       <c r="A187" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="G187" s="9" t="inlineStr"/>
     </row>
-    <row r="188" ht="15" customHeight="1">
+    <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G188" s="5" t="inlineStr"/>
     </row>
-    <row r="189" ht="15" customHeight="1">
+    <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="G189" s="9" t="inlineStr"/>
     </row>
-    <row r="190" ht="15" customHeight="1">
+    <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="G190" s="5" t="inlineStr"/>
     </row>
-    <row r="191" ht="15" customHeight="1">
+    <row r="191">
       <c r="A191" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="G191" s="9" t="inlineStr"/>
     </row>
-    <row r="192" ht="15" customHeight="1">
+    <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6541,7 +6541,7 @@
       </c>
       <c r="G192" s="5" t="inlineStr"/>
     </row>
-    <row r="193" ht="15" customHeight="1">
+    <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="G193" s="9" t="inlineStr"/>
     </row>
-    <row r="194" ht="15" customHeight="1">
+    <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="G194" s="5" t="inlineStr"/>
     </row>
-    <row r="195" ht="15" customHeight="1">
+    <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6640,7 +6640,7 @@
       </c>
       <c r="G195" s="9" t="inlineStr"/>
     </row>
-    <row r="196" ht="15" customHeight="1">
+    <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6673,7 +6673,7 @@
       </c>
       <c r="G196" s="5" t="inlineStr"/>
     </row>
-    <row r="197" ht="15" customHeight="1">
+    <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6706,7 +6706,7 @@
       </c>
       <c r="G197" s="9" t="inlineStr"/>
     </row>
-    <row r="198" ht="15" customHeight="1">
+    <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6739,7 +6739,7 @@
       </c>
       <c r="G198" s="5" t="inlineStr"/>
     </row>
-    <row r="199" ht="15" customHeight="1">
+    <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="G199" s="9" t="inlineStr"/>
     </row>
-    <row r="200" ht="15" customHeight="1">
+    <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6805,7 +6805,7 @@
       </c>
       <c r="G200" s="5" t="inlineStr"/>
     </row>
-    <row r="201" ht="15" customHeight="1">
+    <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="G201" s="9" t="inlineStr"/>
     </row>
-    <row r="202" ht="15" customHeight="1">
+    <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6871,7 +6871,7 @@
       </c>
       <c r="G202" s="5" t="inlineStr"/>
     </row>
-    <row r="203" ht="15" customHeight="1">
+    <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6900,7 +6900,7 @@
       </c>
       <c r="G203" s="9" t="inlineStr"/>
     </row>
-    <row r="204" ht="15" customHeight="1">
+    <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="G204" s="5" t="inlineStr"/>
     </row>
-    <row r="205" ht="15" customHeight="1">
+    <row r="205">
       <c r="A205" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="G205" s="9" t="inlineStr"/>
     </row>
-    <row r="206" ht="15" customHeight="1">
+    <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -6987,7 +6987,7 @@
       </c>
       <c r="G206" s="5" t="inlineStr"/>
     </row>
-    <row r="207" ht="15" customHeight="1">
+    <row r="207">
       <c r="A207" s="6" t="inlineStr">
         <is>
           <t>About</t>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="G207" s="9" t="inlineStr"/>
     </row>
-    <row r="208" ht="15" customHeight="1">
+    <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
           <t>About</t>
@@ -7045,7 +7045,7 @@
       </c>
       <c r="G208" s="5" t="inlineStr"/>
     </row>
-    <row r="209" ht="15" customHeight="1">
+    <row r="209">
       <c r="A209" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="G209" s="9" t="inlineStr"/>
     </row>
-    <row r="210" ht="15" customHeight="1">
+    <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="G210" s="5" t="inlineStr"/>
     </row>
-    <row r="211" ht="15" customHeight="1">
+    <row r="211">
       <c r="A211" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7132,7 +7132,7 @@
       </c>
       <c r="G211" s="9" t="inlineStr"/>
     </row>
-    <row r="212" ht="15" customHeight="1">
+    <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="G212" s="5" t="inlineStr"/>
     </row>
-    <row r="213" ht="15" customHeight="1">
+    <row r="213">
       <c r="A213" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7190,7 +7190,7 @@
       </c>
       <c r="G213" s="9" t="inlineStr"/>
     </row>
-    <row r="214" ht="15" customHeight="1">
+    <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7219,7 +7219,7 @@
       </c>
       <c r="G214" s="5" t="inlineStr"/>
     </row>
-    <row r="215" ht="15" customHeight="1">
+    <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="G215" s="9" t="inlineStr"/>
     </row>
-    <row r="216" ht="15" customHeight="1">
+    <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7277,7 +7277,7 @@
       </c>
       <c r="G216" s="5" t="inlineStr"/>
     </row>
-    <row r="217" ht="15" customHeight="1">
+    <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="G217" s="9" t="inlineStr"/>
     </row>
-    <row r="218" ht="15" customHeight="1">
+    <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7335,7 +7335,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr"/>
     </row>
-    <row r="219" ht="15" customHeight="1">
+    <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7364,7 +7364,7 @@
       </c>
       <c r="G219" s="9" t="inlineStr"/>
     </row>
-    <row r="220" ht="15" customHeight="1">
+    <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7393,7 +7393,7 @@
       </c>
       <c r="G220" s="5" t="inlineStr"/>
     </row>
-    <row r="221" ht="15" customHeight="1">
+    <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7422,7 +7422,7 @@
       </c>
       <c r="G221" s="9" t="inlineStr"/>
     </row>
-    <row r="222" ht="15" customHeight="1">
+    <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7451,7 +7451,7 @@
       </c>
       <c r="G222" s="5" t="inlineStr"/>
     </row>
-    <row r="223" ht="15" customHeight="1">
+    <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="G223" s="9" t="inlineStr"/>
     </row>
-    <row r="224" ht="15" customHeight="1">
+    <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7517,7 +7517,7 @@
       </c>
       <c r="G224" s="5" t="inlineStr"/>
     </row>
-    <row r="225" ht="15" customHeight="1">
+    <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="G225" s="9" t="inlineStr"/>
     </row>
-    <row r="226" ht="15" customHeight="1">
+    <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7583,7 +7583,7 @@
       </c>
       <c r="G226" s="5" t="inlineStr"/>
     </row>
-    <row r="227" ht="15" customHeight="1">
+    <row r="227">
       <c r="A227" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7616,7 +7616,7 @@
       </c>
       <c r="G227" s="9" t="inlineStr"/>
     </row>
-    <row r="228" ht="15" customHeight="1">
+    <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="G228" s="5" t="inlineStr"/>
     </row>
-    <row r="229" ht="15" customHeight="1">
+    <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="G229" s="9" t="inlineStr"/>
     </row>
-    <row r="230" ht="15" customHeight="1">
+    <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7715,7 +7715,7 @@
       </c>
       <c r="G230" s="5" t="inlineStr"/>
     </row>
-    <row r="231" ht="15" customHeight="1">
+    <row r="231">
       <c r="A231" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="G231" s="9" t="inlineStr"/>
     </row>
-    <row r="232" ht="15" customHeight="1">
+    <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="G232" s="5" t="inlineStr"/>
     </row>
-    <row r="233" ht="15" customHeight="1">
+    <row r="233">
       <c r="A233" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="G233" s="9" t="inlineStr"/>
     </row>
-    <row r="234" ht="15" customHeight="1">
+    <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="G234" s="5" t="inlineStr"/>
     </row>
-    <row r="235" ht="15" customHeight="1">
+    <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7860,7 +7860,7 @@
       </c>
       <c r="G235" s="9" t="inlineStr"/>
     </row>
-    <row r="236" ht="15" customHeight="1">
+    <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="G236" s="5" t="inlineStr"/>
     </row>
-    <row r="237" ht="15" customHeight="1">
+    <row r="237">
       <c r="A237" s="6" t="inlineStr">
         <is>
           <t>Contact</t>
@@ -7918,7 +7918,7 @@
       </c>
       <c r="G237" s="9" t="inlineStr"/>
     </row>
-    <row r="238" ht="15" customHeight="1">
+    <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
           <t>Contact</t>

</xml_diff>